<commit_message>
Revise Topics 1 and 2 Excel instruction materials
</commit_message>
<xml_diff>
--- a/docs/unit1/2_lookup_match_if/(Starter-Workbook)-HW-Lookups-Match-IF.xlsx
+++ b/docs/unit1/2_lookup_match_if/(Starter-Workbook)-HW-Lookups-Match-IF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/griffinizu/PycharmProjects/content/docs/unit1/2_lookup_match_if/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\GIT_Repo\CCE_270_content\docs\unit1\2_lookup_match_if\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C9C2122-A379-F544-BCFC-B5A8996D6D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647E2294-589B-4132-8F71-DBC3AA3C6B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24825" yWindow="1545" windowWidth="32775" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hydrometer Analysis" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   <definedNames>
     <definedName name="GravelCosts">Tables!$V$1:$W$6</definedName>
     <definedName name="PricePerTest">Tables!$J$1:$T$9</definedName>
-    <definedName name="StokesLaw">Tables!$A$1:$H$17</definedName>
+    <definedName name="StokesLaw">Tables!$A$4:$H$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="88">
   <si>
     <t>Hydrometer Analysis</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Deflection (v) for x≤a:</t>
   </si>
   <si>
-    <t>[lb/in^2}</t>
-  </si>
-  <si>
     <t>Mom. of Inertia (Iu):</t>
   </si>
   <si>
@@ -301,6 +298,12 @@
   </si>
   <si>
     <t>K</t>
+  </si>
+  <si>
+    <t>[lb/in^2]</t>
+  </si>
+  <si>
+    <t>[in^4]</t>
   </si>
 </sst>
 </file>
@@ -1067,6 +1070,17 @@
     <xf numFmtId="164" fontId="24" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1077,11 +1091,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1090,12 +1099,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1455,21 +1458,21 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
     <col min="3" max="6" width="11" customWidth="1"/>
-    <col min="7" max="13" width="14.5" customWidth="1"/>
+    <col min="7" max="13" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="55" customFormat="1" ht="32" customHeight="1">
-      <c r="A1" s="64" t="s">
+    <row r="1" spans="1:13" s="55" customFormat="1" ht="32.1" customHeight="1">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
       <c r="G1" s="56"/>
       <c r="H1" s="57"/>
       <c r="I1" s="57"/>
@@ -1479,11 +1482,11 @@
       <c r="M1" s="57"/>
     </row>
     <row r="2" spans="1:13" ht="15">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
       <c r="D2" s="53" t="s">
         <v>2</v>
       </c>
@@ -1496,11 +1499,11 @@
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:13" ht="15">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="70"/>
+      <c r="B3" s="65"/>
+      <c r="C3" s="66"/>
       <c r="D3" s="50" t="s">
         <v>6</v>
       </c>
@@ -1513,11 +1516,11 @@
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:13" ht="15">
-      <c r="A4" s="68" t="s">
+      <c r="A4" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="69"/>
-      <c r="C4" s="70"/>
+      <c r="B4" s="65"/>
+      <c r="C4" s="66"/>
       <c r="D4" s="50" t="s">
         <v>9</v>
       </c>
@@ -1528,11 +1531,11 @@
       <c r="G4" s="4"/>
     </row>
     <row r="5" spans="1:13" ht="15">
-      <c r="A5" s="71" t="s">
+      <c r="A5" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="73"/>
+      <c r="B5" s="74"/>
+      <c r="C5" s="75"/>
       <c r="D5" s="50" t="s">
         <v>11</v>
       </c>
@@ -1545,9 +1548,9 @@
       <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:13" ht="15">
-      <c r="A6" s="74"/>
-      <c r="B6" s="75"/>
-      <c r="C6" s="76"/>
+      <c r="A6" s="76"/>
+      <c r="B6" s="77"/>
+      <c r="C6" s="78"/>
       <c r="D6" s="50" t="s">
         <v>13</v>
       </c>
@@ -1558,11 +1561,11 @@
       <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:13" ht="15">
-      <c r="A7" s="68" t="s">
+      <c r="A7" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="69"/>
-      <c r="C7" s="70"/>
+      <c r="B7" s="65"/>
+      <c r="C7" s="66"/>
       <c r="D7" s="50" t="s">
         <v>16</v>
       </c>
@@ -1573,11 +1576,11 @@
       <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:13" ht="15">
-      <c r="A8" s="68" t="s">
+      <c r="A8" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="69"/>
-      <c r="C8" s="70"/>
+      <c r="B8" s="65"/>
+      <c r="C8" s="66"/>
       <c r="D8" s="50" t="s">
         <v>18</v>
       </c>
@@ -1588,11 +1591,11 @@
       <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:13" ht="15">
-      <c r="A9" s="68" t="s">
+      <c r="A9" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="69"/>
-      <c r="C9" s="70"/>
+      <c r="B9" s="65"/>
+      <c r="C9" s="66"/>
       <c r="D9" s="50" t="s">
         <v>20</v>
       </c>
@@ -1602,24 +1605,24 @@
       <c r="I9" s="1"/>
     </row>
     <row r="10" spans="1:13" ht="15">
-      <c r="A10" s="68" t="s">
+      <c r="A10" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="69"/>
-      <c r="C10" s="70"/>
+      <c r="B10" s="65"/>
+      <c r="C10" s="66"/>
       <c r="D10" s="50" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E10" s="50"/>
       <c r="F10" s="52"/>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="1:13" ht="15">
-      <c r="A11" s="68" t="s">
+      <c r="A11" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="69"/>
-      <c r="C11" s="70"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="66"/>
       <c r="D11" s="50" t="s">
         <v>23</v>
       </c>
@@ -1630,26 +1633,26 @@
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="1:13" ht="18" customHeight="1"/>
-    <row r="13" spans="1:13" ht="26" customHeight="1">
-      <c r="A13" s="77" t="s">
+    <row r="13" spans="1:13" ht="26.1" customHeight="1">
+      <c r="A13" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="77" t="s">
+      <c r="B13" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="77" t="s">
+      <c r="C13" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="77" t="s">
+      <c r="D13" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="77" t="s">
+      <c r="E13" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="77" t="s">
+      <c r="F13" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="77" t="s">
+      <c r="G13" s="67" t="s">
         <v>30</v>
       </c>
       <c r="H13" s="1"/>
@@ -1659,14 +1662,14 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
     </row>
-    <row r="14" spans="1:13" ht="7" customHeight="1" thickBot="1">
-      <c r="A14" s="78"/>
-      <c r="B14" s="78"/>
-      <c r="C14" s="78"/>
-      <c r="D14" s="78"/>
-      <c r="E14" s="78"/>
-      <c r="F14" s="78"/>
-      <c r="G14" s="78"/>
+    <row r="14" spans="1:13" ht="6.95" customHeight="1" thickBot="1">
+      <c r="A14" s="68"/>
+      <c r="B14" s="68"/>
+      <c r="C14" s="68"/>
+      <c r="D14" s="68"/>
+      <c r="E14" s="68"/>
+      <c r="F14" s="68"/>
+      <c r="G14" s="68"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -1674,7 +1677,7 @@
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
     </row>
-    <row r="15" spans="1:13" ht="16" thickBot="1">
+    <row r="15" spans="1:13" thickBot="1">
       <c r="A15" s="6">
         <v>0.25</v>
       </c>
@@ -1689,7 +1692,7 @@
       </c>
       <c r="G15" s="25"/>
     </row>
-    <row r="16" spans="1:13" ht="16" thickBot="1">
+    <row r="16" spans="1:13" thickBot="1">
       <c r="A16" s="6">
         <v>0.5</v>
       </c>
@@ -1704,7 +1707,7 @@
       </c>
       <c r="G16" s="28"/>
     </row>
-    <row r="17" spans="1:7" ht="16" thickBot="1">
+    <row r="17" spans="1:7" thickBot="1">
       <c r="A17" s="6">
         <v>1</v>
       </c>
@@ -1719,7 +1722,7 @@
       </c>
       <c r="G17" s="28"/>
     </row>
-    <row r="18" spans="1:7" ht="16" thickBot="1">
+    <row r="18" spans="1:7" thickBot="1">
       <c r="A18" s="6">
         <v>2</v>
       </c>
@@ -1734,7 +1737,7 @@
       </c>
       <c r="G18" s="28"/>
     </row>
-    <row r="19" spans="1:7" ht="16" thickBot="1">
+    <row r="19" spans="1:7" thickBot="1">
       <c r="A19" s="6">
         <v>4</v>
       </c>
@@ -1749,7 +1752,7 @@
       </c>
       <c r="G19" s="28"/>
     </row>
-    <row r="20" spans="1:7" ht="16" thickBot="1">
+    <row r="20" spans="1:7" thickBot="1">
       <c r="A20" s="6">
         <v>8</v>
       </c>
@@ -1764,7 +1767,7 @@
       </c>
       <c r="G20" s="28"/>
     </row>
-    <row r="21" spans="1:7" ht="16" thickBot="1">
+    <row r="21" spans="1:7" thickBot="1">
       <c r="A21" s="6">
         <v>15</v>
       </c>
@@ -1779,7 +1782,7 @@
       </c>
       <c r="G21" s="28"/>
     </row>
-    <row r="22" spans="1:7" ht="16" thickBot="1">
+    <row r="22" spans="1:7" thickBot="1">
       <c r="A22" s="6">
         <v>30</v>
       </c>
@@ -1794,7 +1797,7 @@
       </c>
       <c r="G22" s="28"/>
     </row>
-    <row r="23" spans="1:7" ht="16" thickBot="1">
+    <row r="23" spans="1:7" thickBot="1">
       <c r="A23" s="6">
         <v>60</v>
       </c>
@@ -1809,7 +1812,7 @@
       </c>
       <c r="G23" s="28"/>
     </row>
-    <row r="24" spans="1:7" ht="16" thickBot="1">
+    <row r="24" spans="1:7" thickBot="1">
       <c r="A24" s="6">
         <v>787</v>
       </c>
@@ -1824,7 +1827,7 @@
       </c>
       <c r="G24" s="28"/>
     </row>
-    <row r="25" spans="1:7" ht="16" thickBot="1">
+    <row r="25" spans="1:7" thickBot="1">
       <c r="A25" s="6">
         <v>1459</v>
       </c>
@@ -1868,6 +1871,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C6"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="E13:E14"/>
@@ -1880,11 +1888,6 @@
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="C13:C14"/>
     <mergeCell ref="D13:D14"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1897,17 +1900,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" style="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" style="39" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" style="39" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17" customHeight="1">
+    <row r="1" spans="1:7" ht="17.100000000000001" customHeight="1">
       <c r="A1" s="42" t="s">
         <v>31</v>
       </c>
@@ -1924,13 +1927,13 @@
         <v>35</v>
       </c>
       <c r="F1" s="43" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="G1" s="43" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="13">
+    </row>
+    <row r="2" spans="1:7" ht="12.75">
       <c r="A2" s="40">
         <v>1124</v>
       </c>
@@ -1945,7 +1948,7 @@
       <c r="F2" s="40"/>
       <c r="G2" s="41"/>
     </row>
-    <row r="3" spans="1:7" ht="13">
+    <row r="3" spans="1:7" ht="12.75">
       <c r="A3" s="40">
         <v>1107</v>
       </c>
@@ -1960,7 +1963,7 @@
       <c r="F3" s="40"/>
       <c r="G3" s="40"/>
     </row>
-    <row r="4" spans="1:7" ht="13">
+    <row r="4" spans="1:7" ht="12.75">
       <c r="A4" s="40">
         <v>1163</v>
       </c>
@@ -1975,7 +1978,7 @@
       <c r="F4" s="40"/>
       <c r="G4" s="40"/>
     </row>
-    <row r="5" spans="1:7" ht="13">
+    <row r="5" spans="1:7" ht="12.75">
       <c r="A5" s="40">
         <v>1182</v>
       </c>
@@ -1990,7 +1993,7 @@
       <c r="F5" s="40"/>
       <c r="G5" s="40"/>
     </row>
-    <row r="6" spans="1:7" ht="13">
+    <row r="6" spans="1:7" ht="12.75">
       <c r="A6" s="40">
         <v>1175</v>
       </c>
@@ -2005,7 +2008,7 @@
       <c r="F6" s="40"/>
       <c r="G6" s="41"/>
     </row>
-    <row r="7" spans="1:7" ht="13">
+    <row r="7" spans="1:7" ht="12.75">
       <c r="A7" s="40">
         <v>1049</v>
       </c>
@@ -2020,7 +2023,7 @@
       <c r="F7" s="40"/>
       <c r="G7" s="41"/>
     </row>
-    <row r="8" spans="1:7" ht="13">
+    <row r="8" spans="1:7" ht="12.75">
       <c r="A8" s="40">
         <v>1006</v>
       </c>
@@ -2035,7 +2038,7 @@
       <c r="F8" s="40"/>
       <c r="G8" s="41"/>
     </row>
-    <row r="9" spans="1:7" ht="13">
+    <row r="9" spans="1:7" ht="12.75">
       <c r="A9" s="40">
         <v>1129</v>
       </c>
@@ -2050,7 +2053,7 @@
       <c r="F9" s="40"/>
       <c r="G9" s="41"/>
     </row>
-    <row r="10" spans="1:7" ht="13">
+    <row r="10" spans="1:7" ht="12.75">
       <c r="A10" s="40">
         <v>1236</v>
       </c>
@@ -2065,7 +2068,7 @@
       <c r="F10" s="40"/>
       <c r="G10" s="41"/>
     </row>
-    <row r="11" spans="1:7" ht="13">
+    <row r="11" spans="1:7" ht="12.75">
       <c r="A11" s="40">
         <v>1041</v>
       </c>
@@ -2080,7 +2083,7 @@
       <c r="F11" s="40"/>
       <c r="G11" s="41"/>
     </row>
-    <row r="12" spans="1:7" ht="13">
+    <row r="12" spans="1:7" ht="12.75">
       <c r="A12" s="40">
         <v>1016</v>
       </c>
@@ -2095,7 +2098,7 @@
       <c r="F12" s="40"/>
       <c r="G12" s="41"/>
     </row>
-    <row r="13" spans="1:7" ht="13">
+    <row r="13" spans="1:7" ht="12.75">
       <c r="A13" s="40">
         <v>1195</v>
       </c>
@@ -2110,7 +2113,7 @@
       <c r="F13" s="40"/>
       <c r="G13" s="41"/>
     </row>
-    <row r="14" spans="1:7" ht="13">
+    <row r="14" spans="1:7" ht="12.75">
       <c r="A14" s="40">
         <v>1072</v>
       </c>
@@ -2125,7 +2128,7 @@
       <c r="F14" s="40"/>
       <c r="G14" s="41"/>
     </row>
-    <row r="15" spans="1:7" ht="13">
+    <row r="15" spans="1:7" ht="12.75">
       <c r="A15" s="40">
         <v>1073</v>
       </c>
@@ -2140,7 +2143,7 @@
       <c r="F15" s="40"/>
       <c r="G15" s="41"/>
     </row>
-    <row r="16" spans="1:7" ht="13">
+    <row r="16" spans="1:7" ht="12.75">
       <c r="A16" s="40">
         <v>1101</v>
       </c>
@@ -2155,7 +2158,7 @@
       <c r="F16" s="40"/>
       <c r="G16" s="41"/>
     </row>
-    <row r="17" spans="1:7" ht="13">
+    <row r="17" spans="1:7" ht="12.75">
       <c r="A17" s="40">
         <v>1026</v>
       </c>
@@ -2170,7 +2173,7 @@
       <c r="F17" s="40"/>
       <c r="G17" s="41"/>
     </row>
-    <row r="18" spans="1:7" ht="13">
+    <row r="18" spans="1:7" ht="12.75">
       <c r="A18" s="40">
         <v>1040</v>
       </c>
@@ -2185,7 +2188,7 @@
       <c r="F18" s="40"/>
       <c r="G18" s="41"/>
     </row>
-    <row r="19" spans="1:7" ht="13">
+    <row r="19" spans="1:7" ht="12.75">
       <c r="A19" s="40">
         <v>1126</v>
       </c>
@@ -2200,7 +2203,7 @@
       <c r="F19" s="40"/>
       <c r="G19" s="41"/>
     </row>
-    <row r="20" spans="1:7" ht="13">
+    <row r="20" spans="1:7" ht="12.75">
       <c r="A20" s="40">
         <v>1181</v>
       </c>
@@ -2215,7 +2218,7 @@
       <c r="F20" s="40"/>
       <c r="G20" s="41"/>
     </row>
-    <row r="21" spans="1:7" ht="13">
+    <row r="21" spans="1:7" ht="12.75">
       <c r="A21" s="40">
         <v>1002</v>
       </c>
@@ -2230,7 +2233,7 @@
       <c r="F21" s="40"/>
       <c r="G21" s="41"/>
     </row>
-    <row r="22" spans="1:7" ht="13">
+    <row r="22" spans="1:7" ht="12.75">
       <c r="A22" s="40">
         <v>1166</v>
       </c>
@@ -2245,7 +2248,7 @@
       <c r="F22" s="40"/>
       <c r="G22" s="41"/>
     </row>
-    <row r="23" spans="1:7" ht="13">
+    <row r="23" spans="1:7" ht="12.75">
       <c r="A23" s="40">
         <v>1248</v>
       </c>
@@ -2260,7 +2263,7 @@
       <c r="F23" s="40"/>
       <c r="G23" s="41"/>
     </row>
-    <row r="24" spans="1:7" ht="13">
+    <row r="24" spans="1:7" ht="12.75">
       <c r="A24" s="40">
         <v>1138</v>
       </c>
@@ -2275,7 +2278,7 @@
       <c r="F24" s="40"/>
       <c r="G24" s="41"/>
     </row>
-    <row r="25" spans="1:7" ht="13">
+    <row r="25" spans="1:7" ht="12.75">
       <c r="A25" s="40">
         <v>1256</v>
       </c>
@@ -2290,7 +2293,7 @@
       <c r="F25" s="40"/>
       <c r="G25" s="41"/>
     </row>
-    <row r="26" spans="1:7" ht="13">
+    <row r="26" spans="1:7" ht="12.75">
       <c r="A26" s="40">
         <v>1011</v>
       </c>
@@ -2305,7 +2308,7 @@
       <c r="F26" s="40"/>
       <c r="G26" s="41"/>
     </row>
-    <row r="27" spans="1:7" ht="13">
+    <row r="27" spans="1:7" ht="12.75">
       <c r="A27" s="40">
         <v>1163</v>
       </c>
@@ -2320,7 +2323,7 @@
       <c r="F27" s="40"/>
       <c r="G27" s="41"/>
     </row>
-    <row r="28" spans="1:7" ht="13">
+    <row r="28" spans="1:7" ht="12.75">
       <c r="A28" s="40">
         <v>1002</v>
       </c>
@@ -2335,7 +2338,7 @@
       <c r="F28" s="40"/>
       <c r="G28" s="41"/>
     </row>
-    <row r="29" spans="1:7" ht="13">
+    <row r="29" spans="1:7" ht="12.75">
       <c r="A29" s="40">
         <v>1078</v>
       </c>
@@ -2350,7 +2353,7 @@
       <c r="F29" s="40"/>
       <c r="G29" s="41"/>
     </row>
-    <row r="30" spans="1:7" ht="13">
+    <row r="30" spans="1:7" ht="12.75">
       <c r="A30" s="40">
         <v>1058</v>
       </c>
@@ -2365,7 +2368,7 @@
       <c r="F30" s="40"/>
       <c r="G30" s="41"/>
     </row>
-    <row r="31" spans="1:7" ht="13">
+    <row r="31" spans="1:7" ht="12.75">
       <c r="A31" s="40">
         <v>1135</v>
       </c>
@@ -2380,15 +2383,15 @@
       <c r="F31" s="40"/>
       <c r="G31" s="41"/>
     </row>
-    <row r="33" spans="4:5" ht="13">
+    <row r="33" spans="4:5" ht="12.75">
       <c r="D33" s="44" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E33" s="45"/>
     </row>
     <row r="34" spans="4:5" ht="15.75" customHeight="1">
       <c r="D34" s="44" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E34" s="45"/>
     </row>
@@ -2423,14 +2426,14 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" customWidth="1"/>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="17" customHeight="1">
+    <row r="1" spans="1:3" ht="17.100000000000001" customHeight="1">
       <c r="A1" s="79" t="s">
         <v>44</v>
       </c>
@@ -2527,17 +2530,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606274E6-D00F-4C5B-960E-02503400C7A7}">
   <dimension ref="A1:G40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="25.33203125" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" customWidth="1"/>
     <col min="3" max="6" width="8" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" customWidth="1"/>
+    <col min="7" max="7" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1">
       <c r="A1" s="38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -2566,13 +2569,13 @@
     </row>
     <row r="4" spans="1:7" ht="14.25" customHeight="1">
       <c r="A4" s="33" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B4" s="37">
         <v>5000</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D4" s="31"/>
       <c r="E4" s="31"/>
@@ -2581,14 +2584,14 @@
     </row>
     <row r="5" spans="1:7" ht="14.25" customHeight="1">
       <c r="A5" s="33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" s="37">
         <f>10*10^6</f>
         <v>10000000</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D5" s="31"/>
       <c r="E5" s="31"/>
@@ -2597,7 +2600,7 @@
     </row>
     <row r="6" spans="1:7" ht="14.25" customHeight="1">
       <c r="A6" s="33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="37">
         <v>144</v>
@@ -2612,7 +2615,7 @@
     </row>
     <row r="7" spans="1:7" ht="14.25" customHeight="1">
       <c r="A7" s="33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B7" s="37">
         <v>48</v>
@@ -2627,7 +2630,7 @@
     </row>
     <row r="8" spans="1:7" ht="14.25" customHeight="1">
       <c r="A8" s="33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="37"/>
       <c r="C8" s="31"/>
@@ -2638,7 +2641,7 @@
     </row>
     <row r="9" spans="1:7" ht="14.25" customHeight="1">
       <c r="A9" s="33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="37">
         <v>2</v>
@@ -2653,7 +2656,7 @@
     </row>
     <row r="10" spans="1:7" ht="14.25" customHeight="1">
       <c r="A10" s="33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="37">
         <v>4</v>
@@ -2668,7 +2671,7 @@
     </row>
     <row r="11" spans="1:7" ht="14.25" customHeight="1">
       <c r="A11" s="33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="32"/>
       <c r="C11" s="31" t="s">
@@ -2690,11 +2693,11 @@
     </row>
     <row r="13" spans="1:7" ht="14.25" customHeight="1">
       <c r="A13" s="33" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B13" s="32"/>
       <c r="C13" s="31" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="D13" s="31"/>
       <c r="E13" s="31"/>
@@ -2971,17 +2974,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:W17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="9" width="6.33203125" customWidth="1"/>
-    <col min="10" max="10" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="21" width="6.33203125" customWidth="1"/>
-    <col min="22" max="22" width="14.83203125" customWidth="1"/>
-    <col min="23" max="23" width="8.5" customWidth="1"/>
-    <col min="24" max="26" width="6.33203125" customWidth="1"/>
+    <col min="1" max="9" width="6.28515625" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="21" width="6.28515625" customWidth="1"/>
+    <col min="22" max="22" width="14.85546875" customWidth="1"/>
+    <col min="23" max="23" width="8.42578125" customWidth="1"/>
+    <col min="24" max="26" width="6.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="13">
+    <row r="1" spans="1:23" ht="12.75">
       <c r="A1" s="84" t="s">
         <v>57</v>
       </c>
@@ -2995,20 +2998,20 @@
       <c r="J1" s="86" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="70"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="65"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
+      <c r="T1" s="66"/>
       <c r="V1" s="87" t="s">
         <v>59</v>
       </c>
-      <c r="W1" s="70"/>
+      <c r="W1" s="66"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" customHeight="1">
       <c r="A2" s="11" t="s">
@@ -3017,12 +3020,12 @@
       <c r="B2" s="88" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="70"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="66"/>
       <c r="J2" s="12" t="s">
         <v>32</v>
       </c>
@@ -3734,7 +3737,7 @@
         <v>1.23E-2</v>
       </c>
       <c r="F16" s="22">
-        <v>1.3100000000000001E-2</v>
+        <v>1.21E-2</v>
       </c>
       <c r="G16" s="22">
         <v>1.2E-2</v>

</xml_diff>